<commit_message>
Finished adding data for 2022 experiments
</commit_message>
<xml_diff>
--- a/Data/2022_F013B4_CO_ISSWC/2022_F013B4_CO_ISSWC_SoilAnalysis.xlsx
+++ b/Data/2022_F013B4_CO_ISSWC/2022_F013B4_CO_ISSWC_SoilAnalysis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\mnt\Data1\USDA-ALARC\GIS\PDI project\cottondata\Data\2022_F013B4_CO_ISSWC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19D9A94F-61F8-45F7-89AB-BFD8DF55961C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C6785FA-A936-489F-8F92-E06319810A49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="16500" yWindow="-21090" windowWidth="17805" windowHeight="20370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1881,6 +1881,9 @@
       <c r="A3">
         <v>2022</v>
       </c>
+      <c r="B3">
+        <v>108</v>
+      </c>
       <c r="C3" t="s">
         <v>269</v>
       </c>
@@ -1896,13 +1899,13 @@
       <c r="G3" s="3">
         <v>0.66</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="6">
         <v>1.4</v>
       </c>
-      <c r="I3">
+      <c r="I3" s="6">
         <v>8.1</v>
       </c>
-      <c r="J3">
+      <c r="J3" s="6">
         <v>10</v>
       </c>
       <c r="K3" s="7">
@@ -1940,6 +1943,9 @@
       <c r="A4">
         <v>2022</v>
       </c>
+      <c r="B4">
+        <v>108</v>
+      </c>
       <c r="C4" t="s">
         <v>269</v>
       </c>
@@ -1955,13 +1961,13 @@
       <c r="G4" s="3">
         <v>2.4500000000000002</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="6">
         <v>0.8</v>
       </c>
-      <c r="I4">
+      <c r="I4" s="6">
         <v>23.7</v>
       </c>
-      <c r="J4">
+      <c r="J4" s="6">
         <v>8.3000000000000007</v>
       </c>
       <c r="K4" s="7">
@@ -1999,6 +2005,9 @@
       <c r="A5">
         <v>2022</v>
       </c>
+      <c r="B5">
+        <v>108</v>
+      </c>
       <c r="C5" t="s">
         <v>269</v>
       </c>
@@ -2014,13 +2023,13 @@
       <c r="G5" s="3">
         <v>2.04</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="6">
         <v>0.9</v>
       </c>
-      <c r="I5">
+      <c r="I5" s="6">
         <v>13.2</v>
       </c>
-      <c r="J5">
+      <c r="J5" s="6">
         <v>56.9</v>
       </c>
       <c r="K5" s="7">
@@ -2058,6 +2067,9 @@
       <c r="A6">
         <v>2022</v>
       </c>
+      <c r="B6">
+        <v>108</v>
+      </c>
       <c r="C6" t="s">
         <v>269</v>
       </c>
@@ -2073,13 +2085,13 @@
       <c r="G6" s="3">
         <v>1.22</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="6">
         <v>0.8</v>
       </c>
-      <c r="I6">
+      <c r="I6" s="6">
         <v>5.8</v>
       </c>
-      <c r="J6">
+      <c r="J6" s="6">
         <v>7.5</v>
       </c>
       <c r="K6" s="7">
@@ -2117,6 +2129,9 @@
       <c r="A7">
         <v>2022</v>
       </c>
+      <c r="B7">
+        <v>108</v>
+      </c>
       <c r="C7" t="s">
         <v>269</v>
       </c>
@@ -2132,13 +2147,13 @@
       <c r="G7" s="3">
         <v>0.8</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="6">
         <v>0.8</v>
       </c>
-      <c r="I7">
+      <c r="I7" s="6">
         <v>4.9000000000000004</v>
       </c>
-      <c r="J7">
+      <c r="J7" s="6">
         <v>7.9</v>
       </c>
       <c r="K7" s="7">
@@ -2176,6 +2191,9 @@
       <c r="A8">
         <v>2022</v>
       </c>
+      <c r="B8">
+        <v>108</v>
+      </c>
       <c r="C8" t="s">
         <v>270</v>
       </c>
@@ -2191,13 +2209,13 @@
       <c r="G8" s="3">
         <v>0.89</v>
       </c>
-      <c r="H8">
+      <c r="H8" s="6">
         <v>1.4</v>
       </c>
-      <c r="I8">
+      <c r="I8" s="6">
         <v>8.9</v>
       </c>
-      <c r="J8">
+      <c r="J8" s="6">
         <v>9.4</v>
       </c>
       <c r="K8" s="7">
@@ -2235,6 +2253,9 @@
       <c r="A9">
         <v>2022</v>
       </c>
+      <c r="B9">
+        <v>108</v>
+      </c>
       <c r="C9" t="s">
         <v>270</v>
       </c>
@@ -2250,13 +2271,13 @@
       <c r="G9" s="3">
         <v>1.41</v>
       </c>
-      <c r="H9">
+      <c r="H9" s="6">
         <v>0.9</v>
       </c>
-      <c r="I9">
+      <c r="I9" s="6">
         <v>5.3</v>
       </c>
-      <c r="J9">
+      <c r="J9" s="6">
         <v>8.4</v>
       </c>
       <c r="K9" s="7">
@@ -2294,6 +2315,9 @@
       <c r="A10">
         <v>2022</v>
       </c>
+      <c r="B10">
+        <v>108</v>
+      </c>
       <c r="C10" t="s">
         <v>270</v>
       </c>
@@ -2309,13 +2333,13 @@
       <c r="G10" s="3">
         <v>1.31</v>
       </c>
-      <c r="H10">
+      <c r="H10" s="6">
         <v>1</v>
       </c>
-      <c r="I10">
+      <c r="I10" s="6">
         <v>9.1999999999999993</v>
       </c>
-      <c r="J10">
+      <c r="J10" s="6">
         <v>8.3000000000000007</v>
       </c>
       <c r="K10" s="7">
@@ -2353,6 +2377,9 @@
       <c r="A11">
         <v>2022</v>
       </c>
+      <c r="B11">
+        <v>108</v>
+      </c>
       <c r="C11" t="s">
         <v>270</v>
       </c>
@@ -2368,13 +2395,13 @@
       <c r="G11" s="3">
         <v>0.47</v>
       </c>
-      <c r="H11">
+      <c r="H11" s="6">
         <v>0.6</v>
       </c>
-      <c r="I11">
+      <c r="I11" s="6">
         <v>1.5</v>
       </c>
-      <c r="J11">
+      <c r="J11" s="6">
         <v>8.4</v>
       </c>
       <c r="K11" s="7">
@@ -2412,6 +2439,9 @@
       <c r="A12">
         <v>2022</v>
       </c>
+      <c r="B12">
+        <v>108</v>
+      </c>
       <c r="C12" t="s">
         <v>270</v>
       </c>
@@ -2427,13 +2457,13 @@
       <c r="G12" s="3">
         <v>0.85</v>
       </c>
-      <c r="H12">
+      <c r="H12" s="6">
         <v>0.8</v>
       </c>
-      <c r="I12">
+      <c r="I12" s="6">
         <v>3.3</v>
       </c>
-      <c r="J12">
+      <c r="J12" s="6">
         <v>8.1999999999999993</v>
       </c>
       <c r="K12" s="7">
@@ -2471,6 +2501,9 @@
       <c r="A13">
         <v>2022</v>
       </c>
+      <c r="B13">
+        <v>108</v>
+      </c>
       <c r="C13" t="s">
         <v>271</v>
       </c>
@@ -2486,13 +2519,13 @@
       <c r="G13" s="3">
         <v>0.91</v>
       </c>
-      <c r="H13">
+      <c r="H13" s="6">
         <v>1.3</v>
       </c>
-      <c r="I13">
+      <c r="I13" s="6">
         <v>4.0999999999999996</v>
       </c>
-      <c r="J13">
+      <c r="J13" s="6">
         <v>9.9</v>
       </c>
       <c r="K13" s="7">
@@ -2530,6 +2563,9 @@
       <c r="A14">
         <v>2022</v>
       </c>
+      <c r="B14">
+        <v>108</v>
+      </c>
       <c r="C14" t="s">
         <v>271</v>
       </c>
@@ -2545,13 +2581,13 @@
       <c r="G14" s="3">
         <v>0.87</v>
       </c>
-      <c r="H14">
+      <c r="H14" s="6">
         <v>0.8</v>
       </c>
-      <c r="I14">
+      <c r="I14" s="6">
         <v>5.2</v>
       </c>
-      <c r="J14">
+      <c r="J14" s="6">
         <v>8.1</v>
       </c>
       <c r="K14" s="7">
@@ -2589,6 +2625,9 @@
       <c r="A15">
         <v>2022</v>
       </c>
+      <c r="B15">
+        <v>108</v>
+      </c>
       <c r="C15" t="s">
         <v>271</v>
       </c>
@@ -2604,13 +2643,13 @@
       <c r="G15" s="3">
         <v>0.8</v>
       </c>
-      <c r="H15">
+      <c r="H15" s="6">
         <v>0.6</v>
       </c>
-      <c r="I15">
+      <c r="I15" s="6">
         <v>5</v>
       </c>
-      <c r="J15">
+      <c r="J15" s="6">
         <v>6.5</v>
       </c>
       <c r="K15" s="7">
@@ -2648,6 +2687,9 @@
       <c r="A16">
         <v>2022</v>
       </c>
+      <c r="B16">
+        <v>108</v>
+      </c>
       <c r="C16" t="s">
         <v>271</v>
       </c>
@@ -2663,13 +2705,13 @@
       <c r="G16" s="3">
         <v>1.2</v>
       </c>
-      <c r="H16">
+      <c r="H16" s="6">
         <v>0.9</v>
       </c>
-      <c r="I16">
+      <c r="I16" s="6">
         <v>6.3</v>
       </c>
-      <c r="J16">
+      <c r="J16" s="6">
         <v>7.8</v>
       </c>
       <c r="K16" s="7">
@@ -2707,6 +2749,9 @@
       <c r="A17">
         <v>2022</v>
       </c>
+      <c r="B17">
+        <v>108</v>
+      </c>
       <c r="C17" t="s">
         <v>271</v>
       </c>
@@ -2722,13 +2767,13 @@
       <c r="G17" s="3">
         <v>0.78</v>
       </c>
-      <c r="H17">
+      <c r="H17" s="6">
         <v>0.7</v>
       </c>
-      <c r="I17">
+      <c r="I17" s="6">
         <v>2.8</v>
       </c>
-      <c r="J17">
+      <c r="J17" s="6">
         <v>8.1999999999999993</v>
       </c>
       <c r="K17" s="7">
@@ -2766,6 +2811,9 @@
       <c r="A18">
         <v>2022</v>
       </c>
+      <c r="B18">
+        <v>108</v>
+      </c>
       <c r="C18" t="s">
         <v>272</v>
       </c>
@@ -2781,13 +2829,13 @@
       <c r="G18" s="3">
         <v>0.54</v>
       </c>
-      <c r="H18">
+      <c r="H18" s="6">
         <v>1.4</v>
       </c>
-      <c r="I18">
+      <c r="I18" s="6">
         <v>8.9</v>
       </c>
-      <c r="J18">
+      <c r="J18" s="6">
         <v>8.9</v>
       </c>
       <c r="K18" s="7">
@@ -2825,6 +2873,9 @@
       <c r="A19">
         <v>2022</v>
       </c>
+      <c r="B19">
+        <v>108</v>
+      </c>
       <c r="C19" t="s">
         <v>272</v>
       </c>
@@ -2840,13 +2891,13 @@
       <c r="G19" s="3">
         <v>0.77</v>
       </c>
-      <c r="H19">
+      <c r="H19" s="6">
         <v>0.8</v>
       </c>
-      <c r="I19">
+      <c r="I19" s="6">
         <v>5.5</v>
       </c>
-      <c r="J19">
+      <c r="J19" s="6">
         <v>8.4</v>
       </c>
       <c r="K19" s="7">
@@ -2884,6 +2935,9 @@
       <c r="A20">
         <v>2022</v>
       </c>
+      <c r="B20">
+        <v>108</v>
+      </c>
       <c r="C20" t="s">
         <v>272</v>
       </c>
@@ -2899,13 +2953,13 @@
       <c r="G20" s="3">
         <v>2.42</v>
       </c>
-      <c r="H20">
+      <c r="H20" s="6">
         <v>0.9</v>
       </c>
-      <c r="I20">
+      <c r="I20" s="6">
         <v>5.6</v>
       </c>
-      <c r="J20">
+      <c r="J20" s="6">
         <v>8.1999999999999993</v>
       </c>
       <c r="K20" s="7">
@@ -2943,6 +2997,9 @@
       <c r="A21">
         <v>2022</v>
       </c>
+      <c r="B21">
+        <v>108</v>
+      </c>
       <c r="C21" t="s">
         <v>272</v>
       </c>
@@ -2958,13 +3015,13 @@
       <c r="G21" s="3">
         <v>1.1200000000000001</v>
       </c>
-      <c r="H21">
+      <c r="H21" s="6">
         <v>0.8</v>
       </c>
-      <c r="I21">
+      <c r="I21" s="6">
         <v>8.5</v>
       </c>
-      <c r="J21">
+      <c r="J21" s="6">
         <v>7.9</v>
       </c>
       <c r="K21" s="7">
@@ -3002,6 +3059,9 @@
       <c r="A22">
         <v>2022</v>
       </c>
+      <c r="B22">
+        <v>108</v>
+      </c>
       <c r="C22" t="s">
         <v>272</v>
       </c>
@@ -3017,13 +3077,13 @@
       <c r="G22" s="3">
         <v>0.7</v>
       </c>
-      <c r="H22">
+      <c r="H22" s="6">
         <v>0.8</v>
       </c>
-      <c r="I22">
+      <c r="I22" s="6">
         <v>4.9000000000000004</v>
       </c>
-      <c r="J22">
+      <c r="J22" s="6">
         <v>8</v>
       </c>
       <c r="K22" s="7">
@@ -3061,6 +3121,9 @@
       <c r="A23">
         <v>2022</v>
       </c>
+      <c r="B23">
+        <v>108</v>
+      </c>
       <c r="C23" t="s">
         <v>273</v>
       </c>
@@ -3076,13 +3139,13 @@
       <c r="G23" s="3">
         <v>0.61</v>
       </c>
-      <c r="H23">
+      <c r="H23" s="6">
         <v>1.4</v>
       </c>
-      <c r="I23">
+      <c r="I23" s="6">
         <v>3.1</v>
       </c>
-      <c r="J23">
+      <c r="J23" s="6">
         <v>9.1</v>
       </c>
       <c r="K23" s="7">
@@ -3120,6 +3183,9 @@
       <c r="A24">
         <v>2022</v>
       </c>
+      <c r="B24">
+        <v>108</v>
+      </c>
       <c r="C24" t="s">
         <v>273</v>
       </c>
@@ -3135,13 +3201,13 @@
       <c r="G24" s="3">
         <v>1.1000000000000001</v>
       </c>
-      <c r="H24">
+      <c r="H24" s="6">
         <v>0.8</v>
       </c>
-      <c r="I24">
+      <c r="I24" s="6">
         <v>2.7</v>
       </c>
-      <c r="J24">
+      <c r="J24" s="6">
         <v>8</v>
       </c>
       <c r="K24" s="7">
@@ -3179,6 +3245,9 @@
       <c r="A25">
         <v>2022</v>
       </c>
+      <c r="B25">
+        <v>108</v>
+      </c>
       <c r="C25" t="s">
         <v>273</v>
       </c>
@@ -3194,13 +3263,13 @@
       <c r="G25" s="3">
         <v>2.04</v>
       </c>
-      <c r="H25">
+      <c r="H25" s="6">
         <v>0.9</v>
       </c>
-      <c r="I25">
+      <c r="I25" s="6">
         <v>4.2</v>
       </c>
-      <c r="J25">
+      <c r="J25" s="6">
         <v>8.1</v>
       </c>
       <c r="K25" s="7">
@@ -3238,6 +3307,9 @@
       <c r="A26">
         <v>2022</v>
       </c>
+      <c r="B26">
+        <v>108</v>
+      </c>
       <c r="C26" t="s">
         <v>273</v>
       </c>
@@ -3253,13 +3325,13 @@
       <c r="G26" s="3">
         <v>1.21</v>
       </c>
-      <c r="H26">
+      <c r="H26" s="6">
         <v>1</v>
       </c>
-      <c r="I26">
+      <c r="I26" s="6">
         <v>2.7</v>
       </c>
-      <c r="J26">
+      <c r="J26" s="6">
         <v>8.1</v>
       </c>
       <c r="K26" s="7">
@@ -3297,6 +3369,9 @@
       <c r="A27">
         <v>2022</v>
       </c>
+      <c r="B27">
+        <v>108</v>
+      </c>
       <c r="C27" t="s">
         <v>273</v>
       </c>
@@ -3312,13 +3387,13 @@
       <c r="G27" s="3">
         <v>0.96</v>
       </c>
-      <c r="H27">
+      <c r="H27" s="6">
         <v>1</v>
       </c>
-      <c r="I27">
+      <c r="I27" s="6">
         <v>2.2999999999999998</v>
       </c>
-      <c r="J27">
+      <c r="J27" s="6">
         <v>8.4</v>
       </c>
       <c r="K27" s="7">
@@ -3356,6 +3431,9 @@
       <c r="A28">
         <v>2022</v>
       </c>
+      <c r="B28">
+        <v>108</v>
+      </c>
       <c r="C28" t="s">
         <v>274</v>
       </c>
@@ -3371,13 +3449,13 @@
       <c r="G28" s="3">
         <v>0.49</v>
       </c>
-      <c r="H28">
+      <c r="H28" s="6">
         <v>1.3</v>
       </c>
-      <c r="I28">
+      <c r="I28" s="6">
         <v>7.7</v>
       </c>
-      <c r="J28">
+      <c r="J28" s="6">
         <v>8.6999999999999993</v>
       </c>
       <c r="K28" s="7">
@@ -3415,6 +3493,9 @@
       <c r="A29">
         <v>2022</v>
       </c>
+      <c r="B29">
+        <v>108</v>
+      </c>
       <c r="C29" t="s">
         <v>274</v>
       </c>
@@ -3430,13 +3511,13 @@
       <c r="G29" s="3">
         <v>0.72</v>
       </c>
-      <c r="H29">
+      <c r="H29" s="6">
         <v>0.9</v>
       </c>
-      <c r="I29">
+      <c r="I29" s="6">
         <v>2.8</v>
       </c>
-      <c r="J29">
+      <c r="J29" s="6">
         <v>8</v>
       </c>
       <c r="K29" s="7">
@@ -3474,6 +3555,9 @@
       <c r="A30">
         <v>2022</v>
       </c>
+      <c r="B30">
+        <v>108</v>
+      </c>
       <c r="C30" t="s">
         <v>274</v>
       </c>
@@ -3489,13 +3573,13 @@
       <c r="G30" s="3">
         <v>0.86</v>
       </c>
-      <c r="H30">
+      <c r="H30" s="6">
         <v>0.8</v>
       </c>
-      <c r="I30">
+      <c r="I30" s="6">
         <v>6</v>
       </c>
-      <c r="J30">
+      <c r="J30" s="6">
         <v>8</v>
       </c>
       <c r="K30" s="7">
@@ -3533,6 +3617,9 @@
       <c r="A31">
         <v>2022</v>
       </c>
+      <c r="B31">
+        <v>108</v>
+      </c>
       <c r="C31" t="s">
         <v>274</v>
       </c>
@@ -3548,13 +3635,13 @@
       <c r="G31" s="3">
         <v>1.1499999999999999</v>
       </c>
-      <c r="H31">
+      <c r="H31" s="6">
         <v>0.7</v>
       </c>
-      <c r="I31">
+      <c r="I31" s="6">
         <v>9.1</v>
       </c>
-      <c r="J31">
+      <c r="J31" s="6">
         <v>8.1999999999999993</v>
       </c>
       <c r="K31" s="7">
@@ -3592,6 +3679,9 @@
       <c r="A32">
         <v>2022</v>
       </c>
+      <c r="B32">
+        <v>108</v>
+      </c>
       <c r="C32" t="s">
         <v>274</v>
       </c>
@@ -3607,13 +3697,13 @@
       <c r="G32" s="3">
         <v>1.45</v>
       </c>
-      <c r="H32">
+      <c r="H32" s="6">
         <v>0.9</v>
       </c>
-      <c r="I32">
+      <c r="I32" s="6">
         <v>6.3</v>
       </c>
-      <c r="J32">
+      <c r="J32" s="6">
         <v>8</v>
       </c>
       <c r="K32" s="7">

</xml_diff>

<commit_message>
Modified soil analysis method for 2022 cotton
</commit_message>
<xml_diff>
--- a/Data/2022_F013B4_CO_ISSWC/2022_F013B4_CO_ISSWC_SoilAnalysis.xlsx
+++ b/Data/2022_F013B4_CO_ISSWC/2022_F013B4_CO_ISSWC_SoilAnalysis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\mnt\Data1\USDA-ALARC\GIS\PDI project\cottondata\Data\2022_F013B4_CO_ISSWC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C6785FA-A936-489F-8F92-E06319810A49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B4049BC-6B11-4746-9704-586C016E2292}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16500" yWindow="-21090" windowWidth="17805" windowHeight="20370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="16545" yWindow="-21345" windowWidth="17805" windowHeight="20370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SoilDF" sheetId="2" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="641" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="292">
   <si>
     <t>Kind Of Sample</t>
   </si>
@@ -905,15 +905,19 @@
   </si>
   <si>
     <t>SLCEC</t>
+  </si>
+  <si>
+    <t>SOIL_DATE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="168" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
@@ -1398,7 +1402,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1407,6 +1411,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1762,60 +1767,63 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{806945E5-8549-44EC-9B0A-34CFC97C5A04}">
-  <dimension ref="A1:T32"/>
+  <dimension ref="A1:U32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="E1" t="s">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="F1" t="s">
         <v>18</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>19</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>20</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>27</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>28</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>29</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>30</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>31</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>32</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>33</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>34</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>35</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>36</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>265</v>
       </c>
@@ -1823,1917 +1831,2010 @@
         <v>266</v>
       </c>
       <c r="C2" t="s">
+        <v>291</v>
+      </c>
+      <c r="D2" t="s">
         <v>267</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>268</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>275</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>276</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>277</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>278</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>279</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>280</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>281</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>282</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>283</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>284</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
         <v>285</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
         <v>286</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="R2" t="s">
         <v>287</v>
       </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>288</v>
       </c>
-      <c r="S2" t="s">
+      <c r="T2" t="s">
         <v>289</v>
       </c>
-      <c r="T2" t="s">
+      <c r="U2" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2022</v>
       </c>
       <c r="B3">
         <v>108</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D3" t="s">
         <v>269</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>20</v>
       </c>
-      <c r="E3" s="6">
+      <c r="F3" s="6">
         <v>8.1999999999999993</v>
       </c>
-      <c r="F3" s="6">
+      <c r="G3" s="6">
         <v>7.2</v>
       </c>
-      <c r="G3" s="3">
+      <c r="H3" s="3">
         <v>0.66</v>
       </c>
-      <c r="H3" s="6">
+      <c r="I3" s="6">
         <v>1.4</v>
       </c>
-      <c r="I3" s="6">
+      <c r="J3" s="6">
         <v>8.1</v>
       </c>
-      <c r="J3" s="6">
+      <c r="K3" s="6">
         <v>10</v>
       </c>
-      <c r="K3" s="7">
+      <c r="L3" s="7">
         <v>347</v>
       </c>
-      <c r="L3" s="6">
+      <c r="M3" s="6">
         <v>90</v>
       </c>
-      <c r="M3" s="3">
+      <c r="N3" s="3">
         <v>1.68</v>
       </c>
-      <c r="N3" s="6">
+      <c r="O3" s="6">
         <v>9.1</v>
       </c>
-      <c r="O3" s="6">
+      <c r="P3" s="6">
         <v>14.7</v>
       </c>
-      <c r="P3" s="3">
+      <c r="Q3" s="3">
         <v>3.53</v>
       </c>
-      <c r="Q3" s="7">
+      <c r="R3" s="7">
         <v>2570</v>
       </c>
-      <c r="R3" s="7">
+      <c r="S3" s="7">
         <v>219</v>
       </c>
-      <c r="S3" s="7">
+      <c r="T3" s="7">
         <v>474</v>
       </c>
-      <c r="T3" s="6">
+      <c r="U3" s="6">
         <v>17.600000000000001</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2022</v>
       </c>
       <c r="B4">
         <v>108</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D4" t="s">
         <v>269</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <v>60</v>
       </c>
-      <c r="E4" s="6">
+      <c r="F4" s="6">
         <v>8.1</v>
       </c>
-      <c r="F4" s="6">
+      <c r="G4" s="6">
         <v>7.2</v>
       </c>
-      <c r="G4" s="3">
+      <c r="H4" s="3">
         <v>2.4500000000000002</v>
       </c>
-      <c r="H4" s="6">
+      <c r="I4" s="6">
         <v>0.8</v>
       </c>
-      <c r="I4" s="6">
+      <c r="J4" s="6">
         <v>23.7</v>
       </c>
-      <c r="J4" s="6">
+      <c r="K4" s="6">
         <v>8.3000000000000007</v>
       </c>
-      <c r="K4" s="7">
+      <c r="L4" s="7">
         <v>172</v>
       </c>
-      <c r="L4" s="6">
+      <c r="M4" s="6">
         <v>424.4</v>
       </c>
-      <c r="M4" s="3">
+      <c r="N4" s="3">
         <v>0.68</v>
       </c>
-      <c r="N4" s="6">
+      <c r="O4" s="6">
         <v>6.8</v>
       </c>
-      <c r="O4" s="6">
+      <c r="P4" s="6">
         <v>6.7</v>
       </c>
-      <c r="P4" s="3">
+      <c r="Q4" s="3">
         <v>2.06</v>
       </c>
-      <c r="Q4" s="7">
+      <c r="R4" s="7">
         <v>4111</v>
       </c>
-      <c r="R4" s="7">
+      <c r="S4" s="7">
         <v>282</v>
       </c>
-      <c r="S4" s="7">
+      <c r="T4" s="7">
         <v>891</v>
       </c>
-      <c r="T4" s="6">
+      <c r="U4" s="6">
         <v>27.2</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2022</v>
       </c>
       <c r="B5">
         <v>108</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D5" t="s">
         <v>269</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>100</v>
       </c>
-      <c r="E5" s="6">
+      <c r="F5" s="6">
         <v>8</v>
       </c>
-      <c r="F5" s="6">
+      <c r="G5" s="6">
         <v>7.2</v>
       </c>
-      <c r="G5" s="3">
+      <c r="H5" s="3">
         <v>2.04</v>
       </c>
-      <c r="H5" s="6">
+      <c r="I5" s="6">
         <v>0.9</v>
       </c>
-      <c r="I5" s="6">
+      <c r="J5" s="6">
         <v>13.2</v>
       </c>
-      <c r="J5" s="6">
+      <c r="K5" s="6">
         <v>56.9</v>
       </c>
-      <c r="K5" s="7">
+      <c r="L5" s="7">
         <v>88</v>
       </c>
-      <c r="L5" s="6">
+      <c r="M5" s="6">
         <v>401.5</v>
       </c>
-      <c r="M5" s="3">
+      <c r="N5" s="3">
         <v>0.4</v>
       </c>
-      <c r="N5" s="6">
+      <c r="O5" s="6">
         <v>4.5999999999999996</v>
       </c>
-      <c r="O5" s="6">
+      <c r="P5" s="6">
         <v>3</v>
       </c>
-      <c r="P5" s="3">
+      <c r="Q5" s="3">
         <v>0.83</v>
       </c>
-      <c r="Q5" s="7">
+      <c r="R5" s="7">
         <v>4098</v>
       </c>
-      <c r="R5" s="7">
+      <c r="S5" s="7">
         <v>252</v>
       </c>
-      <c r="S5" s="7">
+      <c r="T5" s="7">
         <v>624</v>
       </c>
-      <c r="T5" s="6">
+      <c r="U5" s="6">
         <v>25.5</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2022</v>
       </c>
       <c r="B6">
         <v>108</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D6" t="s">
         <v>269</v>
       </c>
-      <c r="D6">
+      <c r="E6">
         <v>140</v>
       </c>
-      <c r="E6" s="6">
+      <c r="F6" s="6">
         <v>8.1</v>
       </c>
-      <c r="F6" s="6">
+      <c r="G6" s="6">
         <v>7.2</v>
       </c>
-      <c r="G6" s="3">
+      <c r="H6" s="3">
         <v>1.22</v>
       </c>
-      <c r="H6" s="6">
+      <c r="I6" s="6">
         <v>0.8</v>
       </c>
-      <c r="I6" s="6">
+      <c r="J6" s="6">
         <v>5.8</v>
       </c>
-      <c r="J6" s="6">
+      <c r="K6" s="6">
         <v>7.5</v>
       </c>
-      <c r="K6" s="7">
+      <c r="L6" s="7">
         <v>85</v>
       </c>
-      <c r="L6" s="6">
+      <c r="M6" s="6">
         <v>102.6</v>
       </c>
-      <c r="M6" s="3">
+      <c r="N6" s="3">
         <v>0.46</v>
       </c>
-      <c r="N6" s="6">
+      <c r="O6" s="6">
         <v>3.7</v>
       </c>
-      <c r="O6" s="6">
+      <c r="P6" s="6">
         <v>2</v>
       </c>
-      <c r="P6" s="3">
+      <c r="Q6" s="3">
         <v>0.48</v>
       </c>
-      <c r="Q6" s="7">
+      <c r="R6" s="7">
         <v>3888</v>
       </c>
-      <c r="R6" s="7">
+      <c r="S6" s="7">
         <v>238</v>
       </c>
-      <c r="S6" s="7">
+      <c r="T6" s="7">
         <v>397</v>
       </c>
-      <c r="T6" s="6">
+      <c r="U6" s="6">
         <v>23.4</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2022</v>
       </c>
       <c r="B7">
         <v>108</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D7" t="s">
         <v>269</v>
       </c>
-      <c r="D7">
+      <c r="E7">
         <v>180</v>
       </c>
-      <c r="E7" s="6">
+      <c r="F7" s="6">
         <v>8.1</v>
       </c>
-      <c r="F7" s="6">
+      <c r="G7" s="6">
         <v>7.2</v>
       </c>
-      <c r="G7" s="3">
+      <c r="H7" s="3">
         <v>0.8</v>
       </c>
-      <c r="H7" s="6">
+      <c r="I7" s="6">
         <v>0.8</v>
       </c>
-      <c r="I7" s="6">
+      <c r="J7" s="6">
         <v>4.9000000000000004</v>
       </c>
-      <c r="J7" s="6">
+      <c r="K7" s="6">
         <v>7.9</v>
       </c>
-      <c r="K7" s="7">
+      <c r="L7" s="7">
         <v>84</v>
       </c>
-      <c r="L7" s="6">
+      <c r="M7" s="6">
         <v>75</v>
       </c>
-      <c r="M7" s="3">
+      <c r="N7" s="3">
         <v>0.73</v>
       </c>
-      <c r="N7" s="6">
+      <c r="O7" s="6">
         <v>5.0999999999999996</v>
       </c>
-      <c r="O7" s="6">
+      <c r="P7" s="6">
         <v>3</v>
       </c>
-      <c r="P7" s="3">
+      <c r="Q7" s="3">
         <v>0.56999999999999995</v>
       </c>
-      <c r="Q7" s="7">
+      <c r="R7" s="7">
         <v>3377</v>
       </c>
-      <c r="R7" s="7">
+      <c r="S7" s="7">
         <v>207</v>
       </c>
-      <c r="S7" s="7">
+      <c r="T7" s="7">
         <v>284</v>
       </c>
-      <c r="T7" s="6">
+      <c r="U7" s="6">
         <v>20.100000000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2022</v>
       </c>
       <c r="B8">
         <v>108</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D8" t="s">
         <v>270</v>
       </c>
-      <c r="D8">
+      <c r="E8">
         <v>20</v>
       </c>
-      <c r="E8" s="6">
+      <c r="F8" s="6">
         <v>8.1</v>
       </c>
-      <c r="F8" s="6">
+      <c r="G8" s="6">
         <v>7.2</v>
       </c>
-      <c r="G8" s="3">
+      <c r="H8" s="3">
         <v>0.89</v>
       </c>
-      <c r="H8" s="6">
+      <c r="I8" s="6">
         <v>1.4</v>
       </c>
-      <c r="I8" s="6">
+      <c r="J8" s="6">
         <v>8.9</v>
       </c>
-      <c r="J8" s="6">
+      <c r="K8" s="6">
         <v>9.4</v>
       </c>
-      <c r="K8" s="7">
+      <c r="L8" s="7">
         <v>283</v>
       </c>
-      <c r="L8" s="6">
+      <c r="M8" s="6">
         <v>126.4</v>
       </c>
-      <c r="M8" s="3">
+      <c r="N8" s="3">
         <v>1.61</v>
       </c>
-      <c r="N8" s="6">
+      <c r="O8" s="6">
         <v>10.199999999999999</v>
       </c>
-      <c r="O8" s="6">
+      <c r="P8" s="6">
         <v>14.6</v>
       </c>
-      <c r="P8" s="3">
+      <c r="Q8" s="3">
         <v>3.49</v>
       </c>
-      <c r="Q8" s="7">
+      <c r="R8" s="7">
         <v>2322</v>
       </c>
-      <c r="R8" s="7">
+      <c r="S8" s="7">
         <v>209</v>
       </c>
-      <c r="S8" s="7">
+      <c r="T8" s="7">
         <v>419</v>
       </c>
-      <c r="T8" s="6">
+      <c r="U8" s="6">
         <v>15.9</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2022</v>
       </c>
       <c r="B9">
         <v>108</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D9" t="s">
         <v>270</v>
       </c>
-      <c r="D9">
+      <c r="E9">
         <v>60</v>
       </c>
-      <c r="E9" s="6">
+      <c r="F9" s="6">
         <v>8</v>
       </c>
-      <c r="F9" s="6">
+      <c r="G9" s="6">
         <v>7.2</v>
       </c>
-      <c r="G9" s="3">
+      <c r="H9" s="3">
         <v>1.41</v>
       </c>
-      <c r="H9" s="6">
+      <c r="I9" s="6">
         <v>0.9</v>
       </c>
-      <c r="I9" s="6">
+      <c r="J9" s="6">
         <v>5.3</v>
       </c>
-      <c r="J9" s="6">
+      <c r="K9" s="6">
         <v>8.4</v>
       </c>
-      <c r="K9" s="7">
+      <c r="L9" s="7">
         <v>216</v>
       </c>
-      <c r="L9" s="6">
+      <c r="M9" s="6">
         <v>269</v>
       </c>
-      <c r="M9" s="3">
+      <c r="N9" s="3">
         <v>0.54</v>
       </c>
-      <c r="N9" s="6">
+      <c r="O9" s="6">
         <v>7.6</v>
       </c>
-      <c r="O9" s="6">
+      <c r="P9" s="6">
         <v>8.5</v>
       </c>
-      <c r="P9" s="3">
+      <c r="Q9" s="3">
         <v>2.14</v>
       </c>
-      <c r="Q9" s="7">
+      <c r="R9" s="7">
         <v>3562</v>
       </c>
-      <c r="R9" s="7">
+      <c r="S9" s="7">
         <v>309</v>
       </c>
-      <c r="S9" s="7">
+      <c r="T9" s="7">
         <v>775</v>
       </c>
-      <c r="T9" s="6">
+      <c r="U9" s="6">
         <v>24.3</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2022</v>
       </c>
       <c r="B10">
         <v>108</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D10" t="s">
         <v>270</v>
       </c>
-      <c r="D10">
+      <c r="E10">
         <v>100</v>
       </c>
-      <c r="E10" s="6">
+      <c r="F10" s="6">
         <v>8.1</v>
       </c>
-      <c r="F10" s="6">
+      <c r="G10" s="6">
         <v>7.2</v>
       </c>
-      <c r="G10" s="3">
+      <c r="H10" s="3">
         <v>1.31</v>
       </c>
-      <c r="H10" s="6">
+      <c r="I10" s="6">
         <v>1</v>
       </c>
-      <c r="I10" s="6">
+      <c r="J10" s="6">
         <v>9.1999999999999993</v>
       </c>
-      <c r="J10" s="6">
+      <c r="K10" s="6">
         <v>8.3000000000000007</v>
       </c>
-      <c r="K10" s="7">
+      <c r="L10" s="7">
         <v>138</v>
       </c>
-      <c r="L10" s="6">
+      <c r="M10" s="6">
         <v>277.39999999999998</v>
       </c>
-      <c r="M10" s="3">
+      <c r="N10" s="3">
         <v>0.31</v>
       </c>
-      <c r="N10" s="6">
+      <c r="O10" s="6">
         <v>6.6</v>
       </c>
-      <c r="O10" s="6">
+      <c r="P10" s="6">
         <v>5.0999999999999996</v>
       </c>
-      <c r="P10" s="3">
+      <c r="Q10" s="3">
         <v>1.2</v>
       </c>
-      <c r="Q10" s="7">
+      <c r="R10" s="7">
         <v>4384</v>
       </c>
-      <c r="R10" s="7">
+      <c r="S10" s="7">
         <v>302</v>
       </c>
-      <c r="S10" s="7">
+      <c r="T10" s="7">
         <v>737</v>
       </c>
-      <c r="T10" s="6">
+      <c r="U10" s="6">
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2022</v>
       </c>
       <c r="B11">
         <v>108</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D11" t="s">
         <v>270</v>
       </c>
-      <c r="D11">
+      <c r="E11">
         <v>140</v>
       </c>
-      <c r="E11" s="6">
+      <c r="F11" s="6">
         <v>8.4</v>
       </c>
-      <c r="F11" s="6">
+      <c r="G11" s="6">
         <v>7.2</v>
       </c>
-      <c r="G11" s="3">
+      <c r="H11" s="3">
         <v>0.47</v>
       </c>
-      <c r="H11" s="6">
+      <c r="I11" s="6">
         <v>0.6</v>
       </c>
-      <c r="I11" s="6">
+      <c r="J11" s="6">
         <v>1.5</v>
       </c>
-      <c r="J11" s="6">
+      <c r="K11" s="6">
         <v>8.4</v>
       </c>
-      <c r="K11" s="7">
+      <c r="L11" s="7">
         <v>84</v>
       </c>
-      <c r="L11" s="6">
+      <c r="M11" s="6">
         <v>36.4</v>
       </c>
-      <c r="M11" s="3">
+      <c r="N11" s="3">
         <v>0.45</v>
       </c>
-      <c r="N11" s="6">
+      <c r="O11" s="6">
         <v>5.4</v>
       </c>
-      <c r="O11" s="6">
+      <c r="P11" s="6">
         <v>3.1</v>
       </c>
-      <c r="P11" s="3">
+      <c r="Q11" s="3">
         <v>0.66</v>
       </c>
-      <c r="Q11" s="7">
+      <c r="R11" s="7">
         <v>3375</v>
       </c>
-      <c r="R11" s="7">
+      <c r="S11" s="7">
         <v>186</v>
       </c>
-      <c r="S11" s="7">
+      <c r="T11" s="7">
         <v>273</v>
       </c>
-      <c r="T11" s="6">
+      <c r="U11" s="6">
         <v>19.8</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2022</v>
       </c>
       <c r="B12">
         <v>108</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D12" t="s">
         <v>270</v>
       </c>
-      <c r="D12">
+      <c r="E12">
         <v>180</v>
       </c>
-      <c r="E12" s="6">
+      <c r="F12" s="6">
         <v>8.3000000000000007</v>
       </c>
-      <c r="F12" s="6">
+      <c r="G12" s="6">
         <v>7.2</v>
       </c>
-      <c r="G12" s="3">
+      <c r="H12" s="3">
         <v>0.85</v>
       </c>
-      <c r="H12" s="6">
+      <c r="I12" s="6">
         <v>0.8</v>
       </c>
-      <c r="I12" s="6">
+      <c r="J12" s="6">
         <v>3.3</v>
       </c>
-      <c r="J12" s="6">
+      <c r="K12" s="6">
         <v>8.1999999999999993</v>
       </c>
-      <c r="K12" s="7">
+      <c r="L12" s="7">
         <v>126</v>
       </c>
-      <c r="L12" s="6">
+      <c r="M12" s="6">
         <v>76.599999999999994</v>
       </c>
-      <c r="M12" s="3">
+      <c r="N12" s="3">
         <v>0.32</v>
       </c>
-      <c r="N12" s="6">
+      <c r="O12" s="6">
         <v>5.4</v>
       </c>
-      <c r="O12" s="6">
+      <c r="P12" s="6">
         <v>3.5</v>
       </c>
-      <c r="P12" s="3">
+      <c r="Q12" s="3">
         <v>0.7</v>
       </c>
-      <c r="Q12" s="7">
+      <c r="R12" s="7">
         <v>3966</v>
       </c>
-      <c r="R12" s="7">
+      <c r="S12" s="7">
         <v>278</v>
       </c>
-      <c r="S12" s="7">
+      <c r="T12" s="7">
         <v>506</v>
       </c>
-      <c r="T12" s="6">
+      <c r="U12" s="6">
         <v>24.7</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2022</v>
       </c>
       <c r="B13">
         <v>108</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D13" t="s">
         <v>271</v>
       </c>
-      <c r="D13">
+      <c r="E13">
         <v>20</v>
       </c>
-      <c r="E13" s="6">
+      <c r="F13" s="6">
         <v>8.1</v>
       </c>
-      <c r="F13" s="6">
+      <c r="G13" s="6">
         <v>7.2</v>
       </c>
-      <c r="G13" s="3">
+      <c r="H13" s="3">
         <v>0.91</v>
       </c>
-      <c r="H13" s="6">
+      <c r="I13" s="6">
         <v>1.3</v>
       </c>
-      <c r="I13" s="6">
+      <c r="J13" s="6">
         <v>4.0999999999999996</v>
       </c>
-      <c r="J13" s="6">
+      <c r="K13" s="6">
         <v>9.9</v>
       </c>
-      <c r="K13" s="7">
+      <c r="L13" s="7">
         <v>354</v>
       </c>
-      <c r="L13" s="6">
+      <c r="M13" s="6">
         <v>161.30000000000001</v>
       </c>
-      <c r="M13" s="3">
+      <c r="N13" s="3">
         <v>1.81</v>
       </c>
-      <c r="N13" s="6">
+      <c r="O13" s="6">
         <v>8.6</v>
       </c>
-      <c r="O13" s="6">
+      <c r="P13" s="6">
         <v>15</v>
       </c>
-      <c r="P13" s="3">
+      <c r="Q13" s="3">
         <v>3.2</v>
       </c>
-      <c r="Q13" s="7">
+      <c r="R13" s="7">
         <v>2649</v>
       </c>
-      <c r="R13" s="7">
+      <c r="S13" s="7">
         <v>239</v>
       </c>
-      <c r="S13" s="7">
+      <c r="T13" s="7">
         <v>552</v>
       </c>
-      <c r="T13" s="6">
+      <c r="U13" s="6">
         <v>18.5</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2022</v>
       </c>
       <c r="B14">
         <v>108</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D14" t="s">
         <v>271</v>
       </c>
-      <c r="D14">
+      <c r="E14">
         <v>60</v>
       </c>
-      <c r="E14" s="6">
+      <c r="F14" s="6">
         <v>8.3000000000000007</v>
       </c>
-      <c r="F14" s="6">
+      <c r="G14" s="6">
         <v>7.2</v>
       </c>
-      <c r="G14" s="3">
+      <c r="H14" s="3">
         <v>0.87</v>
       </c>
-      <c r="H14" s="6">
+      <c r="I14" s="6">
         <v>0.8</v>
       </c>
-      <c r="I14" s="6">
+      <c r="J14" s="6">
         <v>5.2</v>
       </c>
-      <c r="J14" s="6">
+      <c r="K14" s="6">
         <v>8.1</v>
       </c>
-      <c r="K14" s="7">
+      <c r="L14" s="7">
         <v>190</v>
       </c>
-      <c r="L14" s="6">
+      <c r="M14" s="6">
         <v>98</v>
       </c>
-      <c r="M14" s="3">
+      <c r="N14" s="3">
         <v>0.78</v>
       </c>
-      <c r="N14" s="6">
+      <c r="O14" s="6">
         <v>7.6</v>
       </c>
-      <c r="O14" s="6">
+      <c r="P14" s="6">
         <v>8.6</v>
       </c>
-      <c r="P14" s="3">
+      <c r="Q14" s="3">
         <v>1.76</v>
       </c>
-      <c r="Q14" s="7">
+      <c r="R14" s="7">
         <v>3219</v>
       </c>
-      <c r="R14" s="7">
+      <c r="S14" s="7">
         <v>212</v>
       </c>
-      <c r="S14" s="7">
+      <c r="T14" s="7">
         <v>548</v>
       </c>
-      <c r="T14" s="6">
+      <c r="U14" s="6">
         <v>20.7</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2022</v>
       </c>
       <c r="B15">
         <v>108</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D15" t="s">
         <v>271</v>
       </c>
-      <c r="D15">
+      <c r="E15">
         <v>100</v>
       </c>
-      <c r="E15" s="6">
+      <c r="F15" s="6">
         <v>8.3000000000000007</v>
       </c>
-      <c r="F15" s="6">
+      <c r="G15" s="6">
         <v>7.2</v>
       </c>
-      <c r="G15" s="3">
+      <c r="H15" s="3">
         <v>0.8</v>
       </c>
-      <c r="H15" s="6">
+      <c r="I15" s="6">
         <v>0.6</v>
       </c>
-      <c r="I15" s="6">
+      <c r="J15" s="6">
         <v>5</v>
       </c>
-      <c r="J15" s="6">
+      <c r="K15" s="6">
         <v>6.5</v>
       </c>
-      <c r="K15" s="7">
+      <c r="L15" s="7">
         <v>176</v>
       </c>
-      <c r="L15" s="6">
+      <c r="M15" s="6">
         <v>100.1</v>
       </c>
-      <c r="M15" s="3">
+      <c r="N15" s="3">
         <v>0.54</v>
       </c>
-      <c r="N15" s="6">
+      <c r="O15" s="6">
         <v>6.3</v>
       </c>
-      <c r="O15" s="6">
+      <c r="P15" s="6">
         <v>6.7</v>
       </c>
-      <c r="P15" s="3">
+      <c r="Q15" s="3">
         <v>1.34</v>
       </c>
-      <c r="Q15" s="7">
+      <c r="R15" s="7">
         <v>3470</v>
       </c>
-      <c r="R15" s="7">
+      <c r="S15" s="7">
         <v>222</v>
       </c>
-      <c r="S15" s="7">
+      <c r="T15" s="7">
         <v>476</v>
       </c>
-      <c r="T15" s="6">
+      <c r="U15" s="6">
         <v>21.7</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2022</v>
       </c>
       <c r="B16">
         <v>108</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D16" t="s">
         <v>271</v>
       </c>
-      <c r="D16">
+      <c r="E16">
         <v>140</v>
       </c>
-      <c r="E16" s="6">
+      <c r="F16" s="6">
         <v>8.1</v>
       </c>
-      <c r="F16" s="6">
+      <c r="G16" s="6">
         <v>7.2</v>
       </c>
-      <c r="G16" s="3">
+      <c r="H16" s="3">
         <v>1.2</v>
       </c>
-      <c r="H16" s="6">
+      <c r="I16" s="6">
         <v>0.9</v>
       </c>
-      <c r="I16" s="6">
+      <c r="J16" s="6">
         <v>6.3</v>
       </c>
-      <c r="J16" s="6">
+      <c r="K16" s="6">
         <v>7.8</v>
       </c>
-      <c r="K16" s="7">
+      <c r="L16" s="7">
         <v>141</v>
       </c>
-      <c r="L16" s="6">
+      <c r="M16" s="6">
         <v>294.8</v>
       </c>
-      <c r="M16" s="3">
+      <c r="N16" s="3">
         <v>0.37</v>
       </c>
-      <c r="N16" s="6">
+      <c r="O16" s="6">
         <v>6.1</v>
       </c>
-      <c r="O16" s="6">
+      <c r="P16" s="6">
         <v>4.4000000000000004</v>
       </c>
-      <c r="P16" s="3">
+      <c r="Q16" s="3">
         <v>0.8</v>
       </c>
-      <c r="Q16" s="7">
+      <c r="R16" s="7">
         <v>4028</v>
       </c>
-      <c r="R16" s="7">
+      <c r="S16" s="7">
         <v>284</v>
       </c>
-      <c r="S16" s="7">
+      <c r="T16" s="7">
         <v>480</v>
       </c>
-      <c r="T16" s="6">
+      <c r="U16" s="6">
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2022</v>
       </c>
       <c r="B17">
         <v>108</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D17" t="s">
         <v>271</v>
       </c>
-      <c r="D17">
+      <c r="E17">
         <v>180</v>
       </c>
-      <c r="E17" s="6">
+      <c r="F17" s="6">
         <v>8.1</v>
       </c>
-      <c r="F17" s="6">
+      <c r="G17" s="6">
         <v>7.2</v>
       </c>
-      <c r="G17" s="3">
+      <c r="H17" s="3">
         <v>0.78</v>
       </c>
-      <c r="H17" s="6">
+      <c r="I17" s="6">
         <v>0.7</v>
       </c>
-      <c r="I17" s="6">
+      <c r="J17" s="6">
         <v>2.8</v>
       </c>
-      <c r="J17" s="6">
+      <c r="K17" s="6">
         <v>8.1999999999999993</v>
       </c>
-      <c r="K17" s="7">
+      <c r="L17" s="7">
         <v>85</v>
       </c>
-      <c r="L17" s="6">
+      <c r="M17" s="6">
         <v>112.7</v>
       </c>
-      <c r="M17" s="3">
+      <c r="N17" s="3">
         <v>0.33</v>
       </c>
-      <c r="N17" s="6">
+      <c r="O17" s="6">
         <v>4.8</v>
       </c>
-      <c r="O17" s="6">
+      <c r="P17" s="6">
         <v>2.6</v>
       </c>
-      <c r="P17" s="3">
+      <c r="Q17" s="3">
         <v>0.48</v>
       </c>
-      <c r="Q17" s="7">
+      <c r="R17" s="7">
         <v>3550</v>
       </c>
-      <c r="R17" s="7">
+      <c r="S17" s="7">
         <v>197</v>
       </c>
-      <c r="S17" s="7">
+      <c r="T17" s="7">
         <v>256</v>
       </c>
-      <c r="T17" s="6">
+      <c r="U17" s="6">
         <v>20.7</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2022</v>
       </c>
       <c r="B18">
         <v>108</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D18" t="s">
         <v>272</v>
       </c>
-      <c r="D18">
+      <c r="E18">
         <v>20</v>
       </c>
-      <c r="E18" s="6">
+      <c r="F18" s="6">
         <v>8.1999999999999993</v>
       </c>
-      <c r="F18" s="6">
+      <c r="G18" s="6">
         <v>7.2</v>
       </c>
-      <c r="G18" s="3">
+      <c r="H18" s="3">
         <v>0.54</v>
       </c>
-      <c r="H18" s="6">
+      <c r="I18" s="6">
         <v>1.4</v>
-      </c>
-      <c r="I18" s="6">
-        <v>8.9</v>
       </c>
       <c r="J18" s="6">
         <v>8.9</v>
       </c>
-      <c r="K18" s="7">
+      <c r="K18" s="6">
+        <v>8.9</v>
+      </c>
+      <c r="L18" s="7">
         <v>277</v>
       </c>
-      <c r="L18" s="6">
+      <c r="M18" s="6">
         <v>63.2</v>
       </c>
-      <c r="M18" s="3">
+      <c r="N18" s="3">
         <v>1.63</v>
       </c>
-      <c r="N18" s="6">
+      <c r="O18" s="6">
         <v>8</v>
       </c>
-      <c r="O18" s="6">
+      <c r="P18" s="6">
         <v>15.9</v>
       </c>
-      <c r="P18" s="3">
+      <c r="Q18" s="3">
         <v>3.37</v>
       </c>
-      <c r="Q18" s="7">
+      <c r="R18" s="7">
         <v>2178</v>
       </c>
-      <c r="R18" s="7">
+      <c r="S18" s="7">
         <v>205</v>
       </c>
-      <c r="S18" s="7">
+      <c r="T18" s="7">
         <v>298</v>
       </c>
-      <c r="T18" s="6">
+      <c r="U18" s="6">
         <v>14.6</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2022</v>
       </c>
       <c r="B19">
         <v>108</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D19" t="s">
         <v>272</v>
       </c>
-      <c r="D19">
+      <c r="E19">
         <v>60</v>
       </c>
-      <c r="E19" s="6">
+      <c r="F19" s="6">
         <v>8.5</v>
       </c>
-      <c r="F19" s="6">
+      <c r="G19" s="6">
         <v>7.2</v>
       </c>
-      <c r="G19" s="3">
+      <c r="H19" s="3">
         <v>0.77</v>
       </c>
-      <c r="H19" s="6">
+      <c r="I19" s="6">
         <v>0.8</v>
       </c>
-      <c r="I19" s="6">
+      <c r="J19" s="6">
         <v>5.5</v>
       </c>
-      <c r="J19" s="6">
+      <c r="K19" s="6">
         <v>8.4</v>
       </c>
-      <c r="K19" s="7">
+      <c r="L19" s="7">
         <v>166</v>
       </c>
-      <c r="L19" s="6">
+      <c r="M19" s="6">
         <v>119</v>
       </c>
-      <c r="M19" s="3">
+      <c r="N19" s="3">
         <v>0.81</v>
       </c>
-      <c r="N19" s="6">
+      <c r="O19" s="6">
         <v>7.4</v>
       </c>
-      <c r="O19" s="6">
+      <c r="P19" s="6">
         <v>8.9</v>
       </c>
-      <c r="P19" s="3">
+      <c r="Q19" s="3">
         <v>2.2200000000000002</v>
       </c>
-      <c r="Q19" s="7">
+      <c r="R19" s="7">
         <v>3600</v>
       </c>
-      <c r="R19" s="7">
+      <c r="S19" s="7">
         <v>228</v>
       </c>
-      <c r="S19" s="7">
+      <c r="T19" s="7">
         <v>608</v>
       </c>
-      <c r="T19" s="6">
+      <c r="U19" s="6">
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2022</v>
       </c>
       <c r="B20">
         <v>108</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D20" t="s">
         <v>272</v>
       </c>
-      <c r="D20">
+      <c r="E20">
         <v>100</v>
       </c>
-      <c r="E20" s="6">
+      <c r="F20" s="6">
         <v>8.1</v>
       </c>
-      <c r="F20" s="6">
+      <c r="G20" s="6">
         <v>7.2</v>
       </c>
-      <c r="G20" s="3">
+      <c r="H20" s="3">
         <v>2.42</v>
       </c>
-      <c r="H20" s="6">
+      <c r="I20" s="6">
         <v>0.9</v>
       </c>
-      <c r="I20" s="6">
+      <c r="J20" s="6">
         <v>5.6</v>
       </c>
-      <c r="J20" s="6">
+      <c r="K20" s="6">
         <v>8.1999999999999993</v>
       </c>
-      <c r="K20" s="7">
+      <c r="L20" s="7">
         <v>120</v>
       </c>
-      <c r="L20" s="6">
+      <c r="M20" s="6">
         <v>368.4</v>
       </c>
-      <c r="M20" s="3">
+      <c r="N20" s="3">
         <v>0.31</v>
       </c>
-      <c r="N20" s="6">
+      <c r="O20" s="6">
         <v>5.9</v>
       </c>
-      <c r="O20" s="6">
+      <c r="P20" s="6">
         <v>3.9</v>
       </c>
-      <c r="P20" s="3">
+      <c r="Q20" s="3">
         <v>0.99</v>
       </c>
-      <c r="Q20" s="7">
+      <c r="R20" s="7">
         <v>4093</v>
       </c>
-      <c r="R20" s="7">
+      <c r="S20" s="7">
         <v>313</v>
       </c>
-      <c r="S20" s="7">
+      <c r="T20" s="7">
         <v>742</v>
       </c>
-      <c r="T20" s="6">
+      <c r="U20" s="6">
         <v>26.6</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2022</v>
       </c>
       <c r="B21">
         <v>108</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D21" t="s">
         <v>272</v>
       </c>
-      <c r="D21">
+      <c r="E21">
         <v>140</v>
       </c>
-      <c r="E21" s="6">
+      <c r="F21" s="6">
         <v>8</v>
       </c>
-      <c r="F21" s="6">
+      <c r="G21" s="6">
         <v>7.2</v>
       </c>
-      <c r="G21" s="3">
+      <c r="H21" s="3">
         <v>1.1200000000000001</v>
       </c>
-      <c r="H21" s="6">
+      <c r="I21" s="6">
         <v>0.8</v>
       </c>
-      <c r="I21" s="6">
+      <c r="J21" s="6">
         <v>8.5</v>
       </c>
-      <c r="J21" s="6">
+      <c r="K21" s="6">
         <v>7.9</v>
       </c>
-      <c r="K21" s="7">
+      <c r="L21" s="7">
         <v>112</v>
       </c>
-      <c r="L21" s="6">
+      <c r="M21" s="6">
         <v>149.1</v>
       </c>
-      <c r="M21" s="3">
+      <c r="N21" s="3">
         <v>0.48</v>
       </c>
-      <c r="N21" s="6">
+      <c r="O21" s="6">
         <v>5.9</v>
       </c>
-      <c r="O21" s="6">
+      <c r="P21" s="6">
         <v>4.8</v>
       </c>
-      <c r="P21" s="3">
+      <c r="Q21" s="3">
         <v>0.94</v>
       </c>
-      <c r="Q21" s="7">
+      <c r="R21" s="7">
         <v>3603</v>
       </c>
-      <c r="R21" s="7">
+      <c r="S21" s="7">
         <v>238</v>
       </c>
-      <c r="S21" s="7">
+      <c r="T21" s="7">
         <v>363</v>
       </c>
-      <c r="T21" s="6">
+      <c r="U21" s="6">
         <v>21.9</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2022</v>
       </c>
       <c r="B22">
         <v>108</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D22" t="s">
         <v>272</v>
       </c>
-      <c r="D22">
+      <c r="E22">
         <v>180</v>
       </c>
-      <c r="E22" s="6">
+      <c r="F22" s="6">
         <v>8.1999999999999993</v>
       </c>
-      <c r="F22" s="6">
+      <c r="G22" s="6">
         <v>7.2</v>
       </c>
-      <c r="G22" s="3">
+      <c r="H22" s="3">
         <v>0.7</v>
       </c>
-      <c r="H22" s="6">
+      <c r="I22" s="6">
         <v>0.8</v>
       </c>
-      <c r="I22" s="6">
+      <c r="J22" s="6">
         <v>4.9000000000000004</v>
       </c>
-      <c r="J22" s="6">
+      <c r="K22" s="6">
         <v>8</v>
       </c>
-      <c r="K22" s="7">
+      <c r="L22" s="7">
         <v>90</v>
       </c>
-      <c r="L22" s="6">
+      <c r="M22" s="6">
         <v>71.7</v>
       </c>
-      <c r="M22" s="3">
+      <c r="N22" s="3">
         <v>0.36</v>
       </c>
-      <c r="N22" s="6">
+      <c r="O22" s="6">
         <v>5.0999999999999996</v>
       </c>
-      <c r="O22" s="6">
+      <c r="P22" s="6">
         <v>3.4</v>
       </c>
-      <c r="P22" s="3">
+      <c r="Q22" s="3">
         <v>0.73</v>
       </c>
-      <c r="Q22" s="7">
+      <c r="R22" s="7">
         <v>3448</v>
       </c>
-      <c r="R22" s="7">
+      <c r="S22" s="7">
         <v>202</v>
       </c>
-      <c r="S22" s="7">
+      <c r="T22" s="7">
         <v>240</v>
       </c>
-      <c r="T22" s="6">
+      <c r="U22" s="6">
         <v>20.2</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2022</v>
       </c>
       <c r="B23">
         <v>108</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D23" t="s">
         <v>273</v>
       </c>
-      <c r="D23">
+      <c r="E23">
         <v>20</v>
       </c>
-      <c r="E23" s="6">
+      <c r="F23" s="6">
         <v>8.1</v>
       </c>
-      <c r="F23" s="6">
+      <c r="G23" s="6">
         <v>7.2</v>
       </c>
-      <c r="G23" s="3">
+      <c r="H23" s="3">
         <v>0.61</v>
       </c>
-      <c r="H23" s="6">
+      <c r="I23" s="6">
         <v>1.4</v>
       </c>
-      <c r="I23" s="6">
+      <c r="J23" s="6">
         <v>3.1</v>
       </c>
-      <c r="J23" s="6">
+      <c r="K23" s="6">
         <v>9.1</v>
       </c>
-      <c r="K23" s="7">
+      <c r="L23" s="7">
         <v>287</v>
       </c>
-      <c r="L23" s="6">
+      <c r="M23" s="6">
         <v>81.599999999999994</v>
       </c>
-      <c r="M23" s="3">
+      <c r="N23" s="3">
         <v>1.43</v>
       </c>
-      <c r="N23" s="6">
+      <c r="O23" s="6">
         <v>8.3000000000000007</v>
       </c>
-      <c r="O23" s="6">
+      <c r="P23" s="6">
         <v>13.6</v>
       </c>
-      <c r="P23" s="3">
+      <c r="Q23" s="3">
         <v>2.93</v>
       </c>
-      <c r="Q23" s="7">
+      <c r="R23" s="7">
         <v>1964</v>
       </c>
-      <c r="R23" s="7">
+      <c r="S23" s="7">
         <v>209</v>
       </c>
-      <c r="S23" s="7">
+      <c r="T23" s="7">
         <v>393</v>
       </c>
-      <c r="T23" s="6">
+      <c r="U23" s="6">
         <v>14</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2022</v>
       </c>
       <c r="B24">
         <v>108</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D24" t="s">
         <v>273</v>
       </c>
-      <c r="D24">
+      <c r="E24">
         <v>60</v>
       </c>
-      <c r="E24" s="6">
+      <c r="F24" s="6">
         <v>8.1999999999999993</v>
       </c>
-      <c r="F24" s="6">
+      <c r="G24" s="6">
         <v>7.2</v>
       </c>
-      <c r="G24" s="3">
+      <c r="H24" s="3">
         <v>1.1000000000000001</v>
       </c>
-      <c r="H24" s="6">
+      <c r="I24" s="6">
         <v>0.8</v>
       </c>
-      <c r="I24" s="6">
+      <c r="J24" s="6">
         <v>2.7</v>
       </c>
-      <c r="J24" s="6">
+      <c r="K24" s="6">
         <v>8</v>
       </c>
-      <c r="K24" s="7">
+      <c r="L24" s="7">
         <v>152</v>
       </c>
-      <c r="L24" s="6">
+      <c r="M24" s="6">
         <v>162.1</v>
       </c>
-      <c r="M24" s="3">
+      <c r="N24" s="3">
         <v>0.4</v>
       </c>
-      <c r="N24" s="6">
+      <c r="O24" s="6">
         <v>7.8</v>
       </c>
-      <c r="O24" s="6">
+      <c r="P24" s="6">
         <v>6.9</v>
       </c>
-      <c r="P24" s="3">
+      <c r="Q24" s="3">
         <v>1.73</v>
       </c>
-      <c r="Q24" s="7">
+      <c r="R24" s="7">
         <v>2985</v>
       </c>
-      <c r="R24" s="7">
+      <c r="S24" s="7">
         <v>237</v>
       </c>
-      <c r="S24" s="7">
+      <c r="T24" s="7">
         <v>675</v>
       </c>
-      <c r="T24" s="6">
+      <c r="U24" s="6">
         <v>20.2</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2022</v>
       </c>
       <c r="B25">
         <v>108</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D25" t="s">
         <v>273</v>
       </c>
-      <c r="D25">
+      <c r="E25">
         <v>100</v>
       </c>
-      <c r="E25" s="6">
+      <c r="F25" s="6">
         <v>8.1</v>
       </c>
-      <c r="F25" s="6">
+      <c r="G25" s="6">
         <v>7.2</v>
       </c>
-      <c r="G25" s="3">
+      <c r="H25" s="3">
         <v>2.04</v>
       </c>
-      <c r="H25" s="6">
+      <c r="I25" s="6">
         <v>0.9</v>
       </c>
-      <c r="I25" s="6">
+      <c r="J25" s="6">
         <v>4.2</v>
       </c>
-      <c r="J25" s="6">
+      <c r="K25" s="6">
         <v>8.1</v>
       </c>
-      <c r="K25" s="7">
+      <c r="L25" s="7">
         <v>136</v>
       </c>
-      <c r="L25" s="6">
+      <c r="M25" s="6">
         <v>183.7</v>
       </c>
-      <c r="M25" s="3">
+      <c r="N25" s="3">
         <v>0.42</v>
       </c>
-      <c r="N25" s="6">
+      <c r="O25" s="6">
         <v>6.5</v>
       </c>
-      <c r="O25" s="6">
+      <c r="P25" s="6">
         <v>5.8</v>
       </c>
-      <c r="P25" s="3">
+      <c r="Q25" s="3">
         <v>1.04</v>
       </c>
-      <c r="Q25" s="7">
+      <c r="R25" s="7">
         <v>3909</v>
       </c>
-      <c r="R25" s="7">
+      <c r="S25" s="7">
         <v>255</v>
       </c>
-      <c r="S25" s="7">
+      <c r="T25" s="7">
         <v>637</v>
       </c>
-      <c r="T25" s="6">
+      <c r="U25" s="6">
         <v>24.8</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2022</v>
       </c>
       <c r="B26">
         <v>108</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D26" t="s">
         <v>273</v>
       </c>
-      <c r="D26">
+      <c r="E26">
         <v>140</v>
       </c>
-      <c r="E26" s="6">
+      <c r="F26" s="6">
         <v>8.1</v>
       </c>
-      <c r="F26" s="6">
+      <c r="G26" s="6">
         <v>7.2</v>
       </c>
-      <c r="G26" s="3">
+      <c r="H26" s="3">
         <v>1.21</v>
       </c>
-      <c r="H26" s="6">
+      <c r="I26" s="6">
         <v>1</v>
       </c>
-      <c r="I26" s="6">
+      <c r="J26" s="6">
         <v>2.7</v>
       </c>
-      <c r="J26" s="6">
+      <c r="K26" s="6">
         <v>8.1</v>
       </c>
-      <c r="K26" s="7">
+      <c r="L26" s="7">
         <v>129</v>
       </c>
-      <c r="L26" s="6">
+      <c r="M26" s="6">
         <v>229.9</v>
       </c>
-      <c r="M26" s="3">
+      <c r="N26" s="3">
         <v>0.35</v>
       </c>
-      <c r="N26" s="6">
+      <c r="O26" s="6">
         <v>9.5</v>
       </c>
-      <c r="O26" s="6">
+      <c r="P26" s="6">
         <v>3.7</v>
       </c>
-      <c r="P26" s="3">
+      <c r="Q26" s="3">
         <v>0.77</v>
       </c>
-      <c r="Q26" s="7">
+      <c r="R26" s="7">
         <v>3955</v>
       </c>
-      <c r="R26" s="7">
+      <c r="S26" s="7">
         <v>282</v>
       </c>
-      <c r="S26" s="7">
+      <c r="T26" s="7">
         <v>456</v>
       </c>
-      <c r="T26" s="6">
+      <c r="U26" s="6">
         <v>24.4</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2022</v>
       </c>
       <c r="B27">
         <v>108</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C27" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D27" t="s">
         <v>273</v>
       </c>
-      <c r="D27">
+      <c r="E27">
         <v>180</v>
       </c>
-      <c r="E27" s="6">
+      <c r="F27" s="6">
         <v>8.1</v>
       </c>
-      <c r="F27" s="6">
+      <c r="G27" s="6">
         <v>7.2</v>
       </c>
-      <c r="G27" s="3">
+      <c r="H27" s="3">
         <v>0.96</v>
       </c>
-      <c r="H27" s="6">
+      <c r="I27" s="6">
         <v>1</v>
       </c>
-      <c r="I27" s="6">
+      <c r="J27" s="6">
         <v>2.2999999999999998</v>
       </c>
-      <c r="J27" s="6">
+      <c r="K27" s="6">
         <v>8.4</v>
       </c>
-      <c r="K27" s="7">
+      <c r="L27" s="7">
         <v>111</v>
       </c>
-      <c r="L27" s="6">
+      <c r="M27" s="6">
         <v>130.6</v>
       </c>
-      <c r="M27" s="3">
+      <c r="N27" s="3">
         <v>0.48</v>
-      </c>
-      <c r="N27" s="6">
-        <v>6.2</v>
       </c>
       <c r="O27" s="6">
         <v>6.2</v>
       </c>
-      <c r="P27" s="3">
+      <c r="P27" s="6">
+        <v>6.2</v>
+      </c>
+      <c r="Q27" s="3">
         <v>0.88</v>
       </c>
-      <c r="Q27" s="7">
+      <c r="R27" s="7">
         <v>3702</v>
       </c>
-      <c r="R27" s="7">
+      <c r="S27" s="7">
         <v>257</v>
       </c>
-      <c r="S27" s="7">
+      <c r="T27" s="7">
         <v>302</v>
       </c>
-      <c r="T27" s="6">
+      <c r="U27" s="6">
         <v>22.2</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>2022</v>
       </c>
       <c r="B28">
         <v>108</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C28" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D28" t="s">
         <v>274</v>
       </c>
-      <c r="D28">
+      <c r="E28">
         <v>20</v>
       </c>
-      <c r="E28" s="6">
+      <c r="F28" s="6">
         <v>8.3000000000000007</v>
       </c>
-      <c r="F28" s="6">
+      <c r="G28" s="6">
         <v>7.2</v>
       </c>
-      <c r="G28" s="3">
+      <c r="H28" s="3">
         <v>0.49</v>
       </c>
-      <c r="H28" s="6">
+      <c r="I28" s="6">
         <v>1.3</v>
       </c>
-      <c r="I28" s="6">
+      <c r="J28" s="6">
         <v>7.7</v>
       </c>
-      <c r="J28" s="6">
+      <c r="K28" s="6">
         <v>8.6999999999999993</v>
       </c>
-      <c r="K28" s="7">
+      <c r="L28" s="7">
         <v>220</v>
       </c>
-      <c r="L28" s="6">
+      <c r="M28" s="6">
         <v>35.4</v>
       </c>
-      <c r="M28" s="3">
+      <c r="N28" s="3">
         <v>1.2</v>
       </c>
-      <c r="N28" s="6">
+      <c r="O28" s="6">
         <v>7.8</v>
       </c>
-      <c r="O28" s="6">
+      <c r="P28" s="6">
         <v>15.5</v>
       </c>
-      <c r="P28" s="3">
+      <c r="Q28" s="3">
         <v>3.02</v>
       </c>
-      <c r="Q28" s="7">
+      <c r="R28" s="7">
         <v>2352</v>
       </c>
-      <c r="R28" s="7">
+      <c r="S28" s="7">
         <v>179</v>
       </c>
-      <c r="S28" s="7">
+      <c r="T28" s="7">
         <v>220</v>
       </c>
-      <c r="T28" s="6">
+      <c r="U28" s="6">
         <v>14.8</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>2022</v>
       </c>
       <c r="B29">
         <v>108</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D29" t="s">
         <v>274</v>
       </c>
-      <c r="D29">
+      <c r="E29">
         <v>60</v>
       </c>
-      <c r="E29" s="6">
+      <c r="F29" s="6">
         <v>8.8000000000000007</v>
       </c>
-      <c r="F29" s="6">
+      <c r="G29" s="6">
         <v>7.2</v>
       </c>
-      <c r="G29" s="3">
+      <c r="H29" s="3">
         <v>0.72</v>
       </c>
-      <c r="H29" s="6">
+      <c r="I29" s="6">
         <v>0.9</v>
       </c>
-      <c r="I29" s="6">
+      <c r="J29" s="6">
         <v>2.8</v>
       </c>
-      <c r="J29" s="6">
+      <c r="K29" s="6">
         <v>8</v>
       </c>
-      <c r="K29" s="7">
+      <c r="L29" s="7">
         <v>99</v>
       </c>
-      <c r="L29" s="6">
+      <c r="M29" s="6">
         <v>43</v>
       </c>
-      <c r="M29" s="3">
+      <c r="N29" s="3">
         <v>0.4</v>
       </c>
-      <c r="N29" s="6">
+      <c r="O29" s="6">
         <v>6.5</v>
       </c>
-      <c r="O29" s="6">
+      <c r="P29" s="6">
         <v>5.2</v>
       </c>
-      <c r="P29" s="3">
+      <c r="Q29" s="3">
         <v>1.43</v>
       </c>
-      <c r="Q29" s="7">
+      <c r="R29" s="7">
         <v>3517</v>
       </c>
-      <c r="R29" s="7">
+      <c r="S29" s="7">
         <v>195</v>
       </c>
-      <c r="S29" s="7">
+      <c r="T29" s="7">
         <v>461</v>
       </c>
-      <c r="T29" s="6">
+      <c r="U29" s="6">
         <v>21.5</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>2022</v>
       </c>
       <c r="B30">
         <v>108</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C30" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D30" t="s">
         <v>274</v>
       </c>
-      <c r="D30">
+      <c r="E30">
         <v>100</v>
       </c>
-      <c r="E30" s="6">
+      <c r="F30" s="6">
         <v>8.8000000000000007</v>
       </c>
-      <c r="F30" s="6">
+      <c r="G30" s="6">
         <v>7.2</v>
       </c>
-      <c r="G30" s="3">
+      <c r="H30" s="3">
         <v>0.86</v>
       </c>
-      <c r="H30" s="6">
+      <c r="I30" s="6">
         <v>0.8</v>
       </c>
-      <c r="I30" s="6">
+      <c r="J30" s="6">
         <v>6</v>
       </c>
-      <c r="J30" s="6">
+      <c r="K30" s="6">
         <v>8</v>
       </c>
-      <c r="K30" s="7">
+      <c r="L30" s="7">
         <v>85</v>
       </c>
-      <c r="L30" s="6">
+      <c r="M30" s="6">
         <v>91.3</v>
       </c>
-      <c r="M30" s="3">
+      <c r="N30" s="3">
         <v>0.3</v>
       </c>
-      <c r="N30" s="6">
+      <c r="O30" s="6">
         <v>5.2</v>
       </c>
-      <c r="O30" s="6">
+      <c r="P30" s="6">
         <v>3.2</v>
       </c>
-      <c r="P30" s="3">
+      <c r="Q30" s="3">
         <v>0.67</v>
       </c>
-      <c r="Q30" s="7">
+      <c r="R30" s="7">
         <v>3517</v>
       </c>
-      <c r="R30" s="7">
+      <c r="S30" s="7">
         <v>186</v>
       </c>
-      <c r="S30" s="7">
+      <c r="T30" s="7">
         <v>469</v>
       </c>
-      <c r="T30" s="6">
+      <c r="U30" s="6">
         <v>21.4</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>2022</v>
       </c>
       <c r="B31">
         <v>108</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D31" t="s">
         <v>274</v>
       </c>
-      <c r="D31">
+      <c r="E31">
         <v>140</v>
       </c>
-      <c r="E31" s="6">
+      <c r="F31" s="6">
         <v>8.4</v>
       </c>
-      <c r="F31" s="6">
+      <c r="G31" s="6">
         <v>7.2</v>
       </c>
-      <c r="G31" s="3">
+      <c r="H31" s="3">
         <v>1.1499999999999999</v>
       </c>
-      <c r="H31" s="6">
+      <c r="I31" s="6">
         <v>0.7</v>
       </c>
-      <c r="I31" s="6">
+      <c r="J31" s="6">
         <v>9.1</v>
       </c>
-      <c r="J31" s="6">
+      <c r="K31" s="6">
         <v>8.1999999999999993</v>
       </c>
-      <c r="K31" s="7">
+      <c r="L31" s="7">
         <v>79</v>
       </c>
-      <c r="L31" s="6">
+      <c r="M31" s="6">
         <v>172.6</v>
       </c>
-      <c r="M31" s="3">
+      <c r="N31" s="3">
         <v>0.16</v>
       </c>
-      <c r="N31" s="6">
+      <c r="O31" s="6">
         <v>4.0999999999999996</v>
       </c>
-      <c r="O31" s="6">
+      <c r="P31" s="6">
         <v>1.9</v>
       </c>
-      <c r="P31" s="3">
+      <c r="Q31" s="3">
         <v>0.36</v>
       </c>
-      <c r="Q31" s="7">
+      <c r="R31" s="7">
         <v>3667</v>
       </c>
-      <c r="R31" s="7">
+      <c r="S31" s="7">
         <v>221</v>
       </c>
-      <c r="S31" s="7">
+      <c r="T31" s="7">
         <v>434</v>
       </c>
-      <c r="T31" s="6">
+      <c r="U31" s="6">
         <v>22.3</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>2022</v>
       </c>
       <c r="B32">
         <v>108</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="8">
+        <v>44669</v>
+      </c>
+      <c r="D32" t="s">
         <v>274</v>
       </c>
-      <c r="D32">
+      <c r="E32">
         <v>180</v>
       </c>
-      <c r="E32" s="6">
+      <c r="F32" s="6">
         <v>8.1</v>
       </c>
-      <c r="F32" s="6">
+      <c r="G32" s="6">
         <v>7.2</v>
       </c>
-      <c r="G32" s="3">
+      <c r="H32" s="3">
         <v>1.45</v>
       </c>
-      <c r="H32" s="6">
+      <c r="I32" s="6">
         <v>0.9</v>
       </c>
-      <c r="I32" s="6">
+      <c r="J32" s="6">
         <v>6.3</v>
       </c>
-      <c r="J32" s="6">
+      <c r="K32" s="6">
         <v>8</v>
       </c>
-      <c r="K32" s="7">
+      <c r="L32" s="7">
         <v>70</v>
       </c>
-      <c r="L32" s="6">
+      <c r="M32" s="6">
         <v>168.6</v>
       </c>
-      <c r="M32" s="3">
+      <c r="N32" s="3">
         <v>0.28999999999999998</v>
       </c>
-      <c r="N32" s="6">
+      <c r="O32" s="6">
         <v>5.0999999999999996</v>
       </c>
-      <c r="O32" s="6">
+      <c r="P32" s="6">
         <v>2.9</v>
       </c>
-      <c r="P32" s="3">
+      <c r="Q32" s="3">
         <v>0.46</v>
       </c>
-      <c r="Q32" s="7">
+      <c r="R32" s="7">
         <v>3620</v>
       </c>
-      <c r="R32" s="7">
+      <c r="S32" s="7">
         <v>205</v>
       </c>
-      <c r="S32" s="7">
+      <c r="T32" s="7">
         <v>287</v>
       </c>
-      <c r="T32" s="6">
+      <c r="U32" s="6">
         <v>21.2</v>
       </c>
     </row>

</xml_diff>